<commit_message>
working towards RawData txt can be saved a tab separated txt from RawData xls or ods sheet
</commit_message>
<xml_diff>
--- a/rawData/RD.xlsx
+++ b/rawData/RD.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DataMSL\Saturation\Daten\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DataSVN\git.GitHub\ahaumer\AppMag\rawData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241C3201-8434-43C0-A816-A25BB4A00730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA89F743-74C1-4B7D-8749-C7AE13A2A82C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{39A8303B-ADE0-4E3B-88E6-F9C4FF7534C2}"/>
   </bookViews>
@@ -455,7 +455,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="26">
   <si>
     <t>M270-50A</t>
   </si>
@@ -464,9 +464,6 @@
   </si>
   <si>
     <t>M400-50A</t>
-  </si>
-  <si>
-    <t>density</t>
   </si>
   <si>
     <t>M310-50A</t>
@@ -499,15 +496,6 @@
     <t>kg/m3</t>
   </si>
   <si>
-    <t>vRef</t>
-  </si>
-  <si>
-    <t>BRef</t>
-  </si>
-  <si>
-    <t>fRef</t>
-  </si>
-  <si>
     <t>W/kg</t>
   </si>
   <si>
@@ -518,9 +506,6 @@
   </si>
   <si>
     <t>N</t>
-  </si>
-  <si>
-    <t>VoestAlpine</t>
   </si>
   <si>
     <t>HP210-35A</t>
@@ -536,6 +521,18 @@
   </si>
   <si>
     <t>CastIron</t>
+  </si>
+  <si>
+    <t># vRef =</t>
+  </si>
+  <si>
+    <t># Bref =</t>
+  </si>
+  <si>
+    <t># fRef =</t>
+  </si>
+  <si>
+    <t># dens =</t>
   </si>
 </sst>
 </file>
@@ -902,56 +899,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7500</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B206)</f>
@@ -960,10 +957,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1203,57 +1200,54 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7700</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B203)</f>
@@ -1262,10 +1256,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1547,59 +1541,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>4.7</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7700</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B202)</f>
@@ -1608,10 +1599,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1893,59 +1884,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>5.3</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7700</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B201)</f>
@@ -1954,10 +1942,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2239,59 +2227,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7750</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B200)</f>
@@ -2300,10 +2285,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2585,59 +2570,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7800</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B199)</f>
@@ -2646,10 +2628,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2931,59 +2913,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7800</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B200)</f>
@@ -2992,10 +2971,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -3277,59 +3256,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>2.1</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7600</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B206)</f>
@@ -3338,10 +3314,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -3623,59 +3599,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>2.35</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7600</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B206)</f>
@@ -3684,10 +3657,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -3969,59 +3942,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>2.5</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7600</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B206)</f>
@@ -4030,10 +4000,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -4315,59 +4285,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>2.7</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7650</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B207)</f>
@@ -4376,10 +4343,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -4663,57 +4630,54 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>2.7</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7600</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B207)</f>
@@ -4722,10 +4686,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -5007,59 +4971,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>3.1</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7650</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B206)</f>
@@ -5068,10 +5029,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -5355,57 +5316,54 @@
       <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>3.3</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7650</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B205)</f>
@@ -5414,10 +5372,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -5699,59 +5657,56 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
         <v>3.5</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>7650</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>COUNT(B8:B205)</f>
@@ -5760,10 +5715,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>